<commit_message>
Add Agent 4 respondent bot, and align its report with Agent 3
</commit_message>
<xml_diff>
--- a/out/S01_campus_cafeteria_experience/agent3/agent3_test_cases_with_paths.xlsx
+++ b/out/S01_campus_cafeteria_experience/agent3/agent3_test_cases_with_paths.xlsx
@@ -5201,22 +5201,22 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Q6 accepts an answer sitting exactly on its stated maximum</t>
+          <t>Q6 blocks a blank answer</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Prove Q6 accepts an answer of exactly 500 characters. A maximum is a limit, so the limit itself is inside the rule. One more than this is already tested as a rejection; an off-by-one in the build sits precisely between the two.</t>
+          <t>Prove Q6 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a text question.</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>A rule that is written down but not enforced lets unusable answers into the data. One that is over-enforced blocks valid respondents.</t>
+          <t>A compulsory question that lets people through blank produces missing data that cannot be recovered afterwards.</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
@@ -5232,12 +5232,12 @@
       <c r="N30" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes
-then: At Q6, type a 500-character answer, then submit.</t>
+then: At Q6, type nothing, then submit.</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>VALID_BOUNDARY (exactly at the limit)</t>
+          <t>EMPTY</t>
         </is>
       </c>
       <c r="P30" s="6" t="inlineStr">
@@ -5247,17 +5247,17 @@
       </c>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>At Q6, type a 500-character answer, then submit.</t>
+          <t>At Q6, type nothing, then submit.</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
         <is>
-          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6 -&gt; Q7 -&gt; Q8</t>
+          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6  (refused at Q6; respondent stays put)</t>
         </is>
       </c>
       <c r="S30" s="6" t="inlineStr">
         <is>
-          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8</t>
+          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6</t>
         </is>
       </c>
       <c r="T30" s="6" t="inlineStr">
@@ -5267,22 +5267,23 @@
       </c>
       <c r="U30" s="6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Q7, Q8</t>
         </is>
       </c>
       <c r="V30" s="6" t="inlineStr">
         <is>
-          <t>Each listed question is followed immediately by the next in the sequence.</t>
+          <t>No forward navigation - the same question must reappear.</t>
         </is>
       </c>
       <c r="W30" s="6" t="inlineStr">
         <is>
-          <t>1. the survey ACCEPTS the answer and moves on</t>
+          <t>1. the survey REFUSES to move on; the same page reappears
+2. an error message is shown against Q6</t>
         </is>
       </c>
       <c r="X30" s="6" t="inlineStr">
         <is>
-          <t>COMPLETE</t>
+          <t>Not reached - the respondent cannot progress</t>
         </is>
       </c>
       <c r="Y30" s="6" t="inlineStr">
@@ -5313,7 +5314,7 @@
       </c>
       <c r="AD30" s="6" t="inlineStr">
         <is>
-          <t>It proves one direction of one rule at one question. The opposite direction is a separate test. It does not prove anything about questions after the one under test, because the journey stops there.</t>
+          <t>It proves only the compulsory setting on this question. Whether the flag is set correctly on other questions is checked separately, question by question.</t>
         </is>
       </c>
       <c r="AE30" s="6" t="inlineStr">
@@ -5343,12 +5344,12 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>2. Input Validation</t>
+          <t>3. Dependency / Piping</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>10. Negative / Robustness</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -5358,22 +5359,22 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Q6 accepts punctuation and quotation marks</t>
+          <t>Q6 quotes the answer given at Q5</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>Prove Q6 accepts an answer containing apostrophes, quotation marks and angle brackets. Its rule constrains length and says nothing about content, so this must be accepted. Quotes and brackets are where survey tools most often break, because nobody wrote the rule down and so nobody tested it.</t>
+          <t>Prove Q6's wording is built from the answer given at Q5, so the respondent is only asked about what they actually chose.</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>A rule that is written down but not enforced lets unusable answers into the data. One that is over-enforced blocks valid respondents.</t>
+          <t>A question that quotes the wrong earlier answer reads as a different question entirely to the respondent.</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -5389,12 +5390,12 @@
       <c r="N31" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes
-then: At Q6, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
+then: At Q6, type “xxxxxxxxxx”, then submit.</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
-          <t>VALID_SPECIAL_CHARACTERS</t>
+          <t>VALID_TYPICAL for every answer</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
@@ -5404,7 +5405,7 @@
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>At Q6, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
+          <t>At Q6, type “xxxxxxxxxx”, then submit.</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -5434,7 +5435,7 @@
       </c>
       <c r="W31" s="6" t="inlineStr">
         <is>
-          <t>1. the survey ACCEPTS the answer and moves on</t>
+          <t>1. Q6's wording includes: Yes</t>
         </is>
       </c>
       <c r="X31" s="6" t="inlineStr">
@@ -5455,7 +5456,7 @@
       </c>
       <c r="AA31" s="6" t="inlineStr">
         <is>
-          <t>Derived by rule from the questionnaire's own tables.</t>
+          <t>QRE explicit - stated directly in the questionnaire.</t>
         </is>
       </c>
       <c r="AB31" s="8" t="inlineStr">
@@ -5470,7 +5471,7 @@
       </c>
       <c r="AD31" s="6" t="inlineStr">
         <is>
-          <t>It proves one direction of one rule at one question. The opposite direction is a separate test. It does not prove anything about questions after the one under test, because the journey stops there.</t>
+          <t>It does not prove anything about questions after the one under test, because the journey stops there.</t>
         </is>
       </c>
       <c r="AE31" s="6" t="inlineStr">
@@ -5500,12 +5501,12 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>2. Input Validation</t>
+          <t>9. Rule Interaction</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>10. Negative / Robustness</t>
+          <t>1. Flow / Routing</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -5515,17 +5516,17 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Q6 refuses an answer of spaces alone</t>
+          <t>Q6 is shown and reflects its dependency on Q5 at the same time</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Prove Q6 refuses an answer of spaces alone. The questionnaire marks it compulsory, and spaces are not an answer. This is the commoner real-world failure than a blank, because a respondent pressing the space bar looks like a respondent who answered.</t>
+          <t>Prove Q6 is shown by its display rule and simultaneously reflects its dependency on Q5. Each mechanism can be correct alone and still disagree together.</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>A compulsory question that lets people through blank produces missing data that cannot be recovered afterwards.</t>
+          <t>Individually correct rules can combine into behaviour neither one describes on its own.</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -5546,12 +5547,12 @@
       <c r="N32" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes
-then: At Q6, type 3 spaces and nothing else, then submit.</t>
+then: At Q6, type “xxxxxxxxxx”, then submit.</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>WHITESPACE_ONLY</t>
+          <t>VALID_TYPICAL for every answer</t>
         </is>
       </c>
       <c r="P32" s="6" t="inlineStr">
@@ -5561,17 +5562,17 @@
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>At Q6, type 3 spaces and nothing else, then submit.</t>
+          <t>At Q6, type “xxxxxxxxxx”, then submit.</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
         <is>
-          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6  (refused at Q6; respondent stays put)</t>
+          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6 -&gt; Q7 -&gt; Q8</t>
         </is>
       </c>
       <c r="S32" s="6" t="inlineStr">
         <is>
-          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6</t>
+          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8</t>
         </is>
       </c>
       <c r="T32" s="6" t="inlineStr">
@@ -5581,23 +5582,23 @@
       </c>
       <c r="U32" s="6" t="inlineStr">
         <is>
-          <t>Q7, Q8</t>
+          <t>none</t>
         </is>
       </c>
       <c r="V32" s="6" t="inlineStr">
         <is>
-          <t>No forward navigation - the same question must reappear.</t>
+          <t>Each listed question is followed immediately by the next in the sequence.</t>
         </is>
       </c>
       <c r="W32" s="6" t="inlineStr">
         <is>
-          <t>1. the survey REFUSES to move on; the same page reappears
-2. an error message is shown against Q6</t>
+          <t>1. Q6 is on screen
+2. Q6's wording includes: Yes</t>
         </is>
       </c>
       <c r="X32" s="6" t="inlineStr">
         <is>
-          <t>Not reached - the respondent cannot progress</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="Y32" s="6" t="inlineStr">
@@ -5613,12 +5614,12 @@
       </c>
       <c r="AA32" s="6" t="inlineStr">
         <is>
-          <t>Derived by rule from the questionnaire's own tables.</t>
-        </is>
-      </c>
-      <c r="AB32" s="10" t="inlineStr">
-        <is>
-          <t>PROVISIONAL</t>
+          <t>QRE explicit - stated directly in the questionnaire.</t>
+        </is>
+      </c>
+      <c r="AB32" s="8" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="AC32" s="8" t="inlineStr">
@@ -5628,12 +5629,12 @@
       </c>
       <c r="AD32" s="6" t="inlineStr">
         <is>
-          <t>It proves only the compulsory setting on this question. Whether the flag is set correctly on other questions is checked separately, question by question.</t>
+          <t>It does not prove anything about questions after the one under test, because the journey stops there.</t>
         </is>
       </c>
       <c r="AE32" s="6" t="inlineStr">
         <is>
-          <t>Leans on an unconfirmed reading: whitespace_is_an_answer</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5664,7 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>10. Negative / Robustness</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -5673,22 +5674,22 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Q6 blocks a blank answer</t>
+          <t>Q6 rejects an invalid answer</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Prove Q6 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a text question.</t>
+          <t>Prove Q6 refuses an answer that breaks its stated rule. The rule is: at least 10 characters; at most 500 characters</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>A compulsory question that lets people through blank produces missing data that cannot be recovered afterwards.</t>
+          <t>A rule that is written down but not enforced lets unusable answers into the data. One that is over-enforced blocks valid respondents.</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr">
@@ -5704,12 +5705,12 @@
       <c r="N33" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes
-then: At Q6, type nothing, then submit.</t>
+then: At Q6, type a 500-character answer, then submit.</t>
         </is>
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
-          <t>EMPTY</t>
+          <t>VALID_TYPICAL for every answer</t>
         </is>
       </c>
       <c r="P33" s="6" t="inlineStr">
@@ -5719,17 +5720,17 @@
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>At Q6, type nothing, then submit.</t>
+          <t>At Q6, type a 500-character answer, then submit.</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
         <is>
-          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6  (refused at Q6; respondent stays put)</t>
+          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6 -&gt; Q7 -&gt; Q8</t>
         </is>
       </c>
       <c r="S33" s="6" t="inlineStr">
         <is>
-          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6</t>
+          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8</t>
         </is>
       </c>
       <c r="T33" s="6" t="inlineStr">
@@ -5739,23 +5740,22 @@
       </c>
       <c r="U33" s="6" t="inlineStr">
         <is>
-          <t>Q7, Q8</t>
+          <t>none</t>
         </is>
       </c>
       <c r="V33" s="6" t="inlineStr">
         <is>
-          <t>No forward navigation - the same question must reappear.</t>
+          <t>Each listed question is followed immediately by the next in the sequence.</t>
         </is>
       </c>
       <c r="W33" s="6" t="inlineStr">
         <is>
-          <t>1. the survey REFUSES to move on; the same page reappears
-2. an error message is shown against Q6</t>
+          <t>1. the survey ACCEPTS the answer and moves on</t>
         </is>
       </c>
       <c r="X33" s="6" t="inlineStr">
         <is>
-          <t>Not reached - the respondent cannot progress</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="Y33" s="6" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="AD33" s="6" t="inlineStr">
         <is>
-          <t>It proves only the compulsory setting on this question. Whether the flag is set correctly on other questions is checked separately, question by question.</t>
+          <t>It proves one direction of one rule at one question. The opposite direction is a separate test. It does not prove anything about questions after the one under test, because the journey stops there.</t>
         </is>
       </c>
       <c r="AE33" s="6" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>3. Dependency / Piping</t>
+          <t>2. Input Validation</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -5831,22 +5831,22 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Q6 quotes the answer given at Q5</t>
+          <t>Q6 rejects an invalid answer</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Prove Q6's wording is built from the answer given at Q5, so the respondent is only asked about what they actually chose.</t>
+          <t>Prove Q6 refuses an answer that breaks its stated rule. The rule is: at least 10 characters; at most 500 characters</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>A question that quotes the wrong earlier answer reads as a different question entirely to the respondent.</t>
+          <t>A rule that is written down but not enforced lets unusable answers into the data. One that is over-enforced blocks valid respondents.</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -5862,7 +5862,7 @@
       <c r="N34" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes
-then: At Q6, type “xxxxxxxxxx”, then submit.</t>
+then: At Q6, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
         </is>
       </c>
       <c r="O34" s="6" t="inlineStr">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>At Q6, type “xxxxxxxxxx”, then submit.</t>
+          <t>At Q6, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="W34" s="6" t="inlineStr">
         <is>
-          <t>1. Q6's wording includes: Yes</t>
+          <t>1. the survey ACCEPTS the answer and moves on</t>
         </is>
       </c>
       <c r="X34" s="6" t="inlineStr">
@@ -5928,7 +5928,7 @@
       </c>
       <c r="AA34" s="6" t="inlineStr">
         <is>
-          <t>QRE explicit - stated directly in the questionnaire.</t>
+          <t>Derived by rule from the questionnaire's own tables.</t>
         </is>
       </c>
       <c r="AB34" s="8" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="AD34" s="6" t="inlineStr">
         <is>
-          <t>It does not prove anything about questions after the one under test, because the journey stops there.</t>
+          <t>It proves one direction of one rule at one question. The opposite direction is a separate test. It does not prove anything about questions after the one under test, because the journey stops there.</t>
         </is>
       </c>
       <c r="AE34" s="6" t="inlineStr">
@@ -5973,12 +5973,12 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>9. Rule Interaction</t>
+          <t>2. Input Validation</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>1. Flow / Routing</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -5988,17 +5988,17 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Q6 is shown and reflects its dependency on Q5 at the same time</t>
+          <t>Q6 allows a blank answer, being optional</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>Prove Q6 is shown by its display rule and simultaneously reflects its dependency on Q5. Each mechanism can be correct alone and still disagree together.</t>
+          <t>Prove Q6 lets the respondent through with no answer, because the questionnaire marks it optional.</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>Individually correct rules can combine into behaviour neither one describes on its own.</t>
+          <t>A compulsory question that lets people through blank produces missing data that cannot be recovered afterwards.</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -6019,7 +6019,7 @@
       <c r="N35" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes
-then: At Q6, type “xxxxxxxxxx”, then submit.</t>
+then: At Q6, type 3 spaces and nothing else, then submit.</t>
         </is>
       </c>
       <c r="O35" s="6" t="inlineStr">
@@ -6034,17 +6034,17 @@
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>At Q6, type “xxxxxxxxxx”, then submit.</t>
+          <t>At Q6, type 3 spaces and nothing else, then submit.</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
         <is>
-          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6 -&gt; Q7 -&gt; Q8</t>
+          <t>S1 -&gt; S2 -&gt; Q1 -&gt; Q2 -&gt; Q3 -&gt; Q4 -&gt; Q5 -&gt; Q6  (refused at Q6; respondent stays put)</t>
         </is>
       </c>
       <c r="S35" s="6" t="inlineStr">
         <is>
-          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8</t>
+          <t>S1, S2, Q1, Q2, Q3, Q4, Q5, Q6</t>
         </is>
       </c>
       <c r="T35" s="6" t="inlineStr">
@@ -6054,23 +6054,23 @@
       </c>
       <c r="U35" s="6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Q7, Q8</t>
         </is>
       </c>
       <c r="V35" s="6" t="inlineStr">
         <is>
-          <t>Each listed question is followed immediately by the next in the sequence.</t>
+          <t>No forward navigation - the same question must reappear.</t>
         </is>
       </c>
       <c r="W35" s="6" t="inlineStr">
         <is>
-          <t>1. Q6 is on screen
-2. Q6's wording includes: Yes</t>
+          <t>1. the survey REFUSES to move on; the same page reappears
+2. an error message is shown against Q6</t>
         </is>
       </c>
       <c r="X35" s="6" t="inlineStr">
         <is>
-          <t>COMPLETE</t>
+          <t>Not reached - the respondent cannot progress</t>
         </is>
       </c>
       <c r="Y35" s="6" t="inlineStr">
@@ -6086,12 +6086,12 @@
       </c>
       <c r="AA35" s="6" t="inlineStr">
         <is>
-          <t>QRE explicit - stated directly in the questionnaire.</t>
-        </is>
-      </c>
-      <c r="AB35" s="8" t="inlineStr">
-        <is>
-          <t>RESOLVED</t>
+          <t>Derived by rule from the questionnaire's own tables.</t>
+        </is>
+      </c>
+      <c r="AB35" s="10" t="inlineStr">
+        <is>
+          <t>PROVISIONAL</t>
         </is>
       </c>
       <c r="AC35" s="8" t="inlineStr">
@@ -6101,12 +6101,12 @@
       </c>
       <c r="AD35" s="6" t="inlineStr">
         <is>
-          <t>It does not prove anything about questions after the one under test, because the journey stops there.</t>
+          <t>It proves only the compulsory setting on this question. Whether the flag is set correctly on other questions is checked separately, question by question.</t>
         </is>
       </c>
       <c r="AE35" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Leans on an unconfirmed reading: whitespace_is_an_answer</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>10. Negative / Robustness</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -6933,22 +6933,22 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Q8 accepts an answer sitting exactly on its stated maximum</t>
+          <t>Q8 allows a blank answer, being optional</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>Prove Q8 accepts an answer of exactly 500 characters. A maximum is a limit, so the limit itself is inside the rule. One more than this is already tested as a rejection; an off-by-one in the build sits precisely between the two.</t>
+          <t>Prove Q8 lets the respondent through with no answer, because the questionnaire marks it optional.</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>A rule that is written down but not enforced lets unusable answers into the data. One that is over-enforced blocks valid respondents.</t>
+          <t>A compulsory question that lets people through blank produces missing data that cannot be recovered afterwards.</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr">
@@ -6964,12 +6964,12 @@
       <c r="N41" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes; Q6 = xxxxxxxxxx; Q7 = 0
-then: At Q8, type a 500-character answer, then submit.</t>
+then: At Q8, type nothing, then submit.</t>
         </is>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
-          <t>VALID_BOUNDARY (exactly at the limit)</t>
+          <t>EMPTY</t>
         </is>
       </c>
       <c r="P41" s="6" t="inlineStr">
@@ -6979,7 +6979,7 @@
       </c>
       <c r="Q41" s="6" t="inlineStr">
         <is>
-          <t>At Q8, type a 500-character answer, then submit.</t>
+          <t>At Q8, type nothing, then submit.</t>
         </is>
       </c>
       <c r="R41" s="6" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="AD41" s="6" t="inlineStr">
         <is>
-          <t>It proves one direction of one rule at one question. The opposite direction is a separate test. It does not prove anything about questions after the one under test, because the journey stops there.</t>
+          <t>It proves only the compulsory setting on this question. Whether the flag is set correctly on other questions is checked separately, question by question.</t>
         </is>
       </c>
       <c r="AE41" s="6" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>10. Negative / Robustness</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -7090,12 +7090,12 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>Q8 accepts punctuation and quotation marks</t>
+          <t>Q8 rejects an invalid answer</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>Prove Q8 accepts an answer containing apostrophes, quotation marks and angle brackets. Its rule constrains length and says nothing about content, so this must be accepted. Quotes and brackets are where survey tools most often break, because nobody wrote the rule down and so nobody tested it.</t>
+          <t>Prove Q8 refuses an answer that breaks its stated rule. The rule is: at most 500 characters</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
@@ -7121,12 +7121,12 @@
       <c r="N42" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes; Q6 = xxxxxxxxxx; Q7 = 0
-then: At Q8, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
+then: At Q8, type a 500-character answer, then submit.</t>
         </is>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
-          <t>VALID_SPECIAL_CHARACTERS</t>
+          <t>VALID_TYPICAL for every answer</t>
         </is>
       </c>
       <c r="P42" s="6" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="Q42" s="6" t="inlineStr">
         <is>
-          <t>At Q8, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
+          <t>At Q8, type a 500-character answer, then submit.</t>
         </is>
       </c>
       <c r="R42" s="6" t="inlineStr">
@@ -7247,22 +7247,22 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Q8 accepts spaces alone, being optional</t>
+          <t>Q8 rejects an invalid answer</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>Prove Q8 accepts an answer of spaces alone. The questionnaire marks it optional, so nothing about the response may block progress.</t>
+          <t>Prove Q8 refuses an answer that breaks its stated rule. The rule is: at most 500 characters</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>A compulsory question that lets people through blank produces missing data that cannot be recovered afterwards.</t>
+          <t>A rule that is written down but not enforced lets unusable answers into the data. One that is over-enforced blocks valid respondents.</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L43" s="6" t="inlineStr">
@@ -7278,12 +7278,12 @@
       <c r="N43" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes; Q6 = xxxxxxxxxx; Q7 = 0
-then: At Q8, type 3 spaces and nothing else, then submit.</t>
+then: At Q8, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
         </is>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
-          <t>WHITESPACE_ONLY</t>
+          <t>VALID_TYPICAL for every answer</t>
         </is>
       </c>
       <c r="P43" s="6" t="inlineStr">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>At Q8, type 3 spaces and nothing else, then submit.</t>
+          <t>At Q8, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
@@ -7347,9 +7347,9 @@
           <t>QRE explicit - stated directly in the questionnaire.</t>
         </is>
       </c>
-      <c r="AB43" s="10" t="inlineStr">
-        <is>
-          <t>PROVISIONAL</t>
+      <c r="AB43" s="8" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="AC43" s="8" t="inlineStr">
@@ -7359,12 +7359,12 @@
       </c>
       <c r="AD43" s="6" t="inlineStr">
         <is>
-          <t>It proves only the compulsory setting on this question. Whether the flag is set correctly on other questions is checked separately, question by question.</t>
+          <t>It proves one direction of one rule at one question. The opposite direction is a separate test. It does not prove anything about questions after the one under test, because the journey stops there.</t>
         </is>
       </c>
       <c r="AE43" s="6" t="inlineStr">
         <is>
-          <t>Leans on an unconfirmed reading: whitespace_is_an_answer</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -7435,12 +7435,12 @@
       <c r="N44" s="6" t="inlineStr">
         <is>
           <t>S1 = Yes; S2 = Yes; Q1 = Counter; Q2 = Very poor; Q3 = Very poor; Q4 = Food quality; Q5 = Yes; Q6 = xxxxxxxxxx; Q7 = 0
-then: At Q8, type nothing, then submit.</t>
+then: At Q8, type 3 spaces and nothing else, then submit.</t>
         </is>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
-          <t>EMPTY</t>
+          <t>VALID_TYPICAL for every answer</t>
         </is>
       </c>
       <c r="P44" s="6" t="inlineStr">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="Q44" s="6" t="inlineStr">
         <is>
-          <t>At Q8, type nothing, then submit.</t>
+          <t>At Q8, type 3 spaces and nothing else, then submit.</t>
         </is>
       </c>
       <c r="R44" s="6" t="inlineStr">
@@ -7504,9 +7504,9 @@
           <t>QRE explicit - stated directly in the questionnaire.</t>
         </is>
       </c>
-      <c r="AB44" s="8" t="inlineStr">
-        <is>
-          <t>RESOLVED</t>
+      <c r="AB44" s="10" t="inlineStr">
+        <is>
+          <t>PROVISIONAL</t>
         </is>
       </c>
       <c r="AC44" s="8" t="inlineStr">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="AE44" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Leans on an unconfirmed reading: whitespace_is_an_answer</t>
         </is>
       </c>
     </row>

</xml_diff>